<commit_message>
test: regenerate Sheets.xlsx fixture for corrected brk@max
</commit_message>
<xml_diff>
--- a/XLibur.Tests/Resource/Examples/PageSetup/Sheets.xlsx
+++ b/XLibur.Tests/Resource/Examples/PageSetup/Sheets.xlsx
@@ -391,10 +391,10 @@
   <x:pageSetup paperSize="1" scale="100" pageOrder="downThenOver" orientation="default" blackAndWhite="0" draft="0" cellComments="none" errors="displayed"/>
   <x:headerFooter/>
   <x:rowBreaks count="1" manualBreakCount="1">
-    <x:brk id="2" max="1048576" man="1"/>
+    <x:brk id="2" max="16383" man="1"/>
   </x:rowBreaks>
   <x:colBreaks count="1" manualBreakCount="1">
-    <x:brk id="2" max="16384" man="1"/>
+    <x:brk id="2" max="1048575" man="1"/>
   </x:colBreaks>
   <x:tableParts count="0"/>
 </x:worksheet>

</xml_diff>

<commit_message>
fix: write correct brk@max extent for page breaks (ClosedXML #2842) (#157)
* fix: write correct brk@max extent for page breaks

A <brk> element's max attribute is the extent perpendicular to the
break: a row (horizontal) break spans the full column width, and a
column (vertical) break spans the full row height. Both were inverted,
writing their own axis extent instead.

Row breaks wrote max=1048576 (the sheet row count), which Excel treats
as a giant used range and renders an abnormally long vertical scrollbar.
Column breaks had the mirror-image defect (max=16384). Now row breaks
write the last column (16383, XFD) and column breaks write the last row
(1048575), matching Excel's own output.

Inherited verbatim from ClosedXML; see ClosedXML issue #2842.

* test: regenerate Sheets.xlsx fixture for corrected brk@max
</commit_message>
<xml_diff>
--- a/XLibur.Tests/Resource/Examples/PageSetup/Sheets.xlsx
+++ b/XLibur.Tests/Resource/Examples/PageSetup/Sheets.xlsx
@@ -391,10 +391,10 @@
   <x:pageSetup paperSize="1" scale="100" pageOrder="downThenOver" orientation="default" blackAndWhite="0" draft="0" cellComments="none" errors="displayed"/>
   <x:headerFooter/>
   <x:rowBreaks count="1" manualBreakCount="1">
-    <x:brk id="2" max="1048576" man="1"/>
+    <x:brk id="2" max="16383" man="1"/>
   </x:rowBreaks>
   <x:colBreaks count="1" manualBreakCount="1">
-    <x:brk id="2" max="16384" man="1"/>
+    <x:brk id="2" max="1048575" man="1"/>
   </x:colBreaks>
   <x:tableParts count="0"/>
 </x:worksheet>

</xml_diff>